<commit_message>
Updated to reflect the micro servo update
</commit_message>
<xml_diff>
--- a/Coursework/Battery Life Calculator.xlsx
+++ b/Coursework/Battery Life Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\RDD Course\Coursework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1725EFBB-00E7-4F7B-8D09-313B34929EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BFA1A9-20C9-4230-A309-509487035D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6480" yWindow="2025" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Item #</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>Total Operation Duration</t>
+  </si>
+  <si>
+    <t>SG90 MicroServo</t>
   </si>
 </sst>
 </file>
@@ -778,11 +781,11 @@
         <v>24</v>
       </c>
       <c r="F2" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2" s="10">
         <f t="shared" ref="G2:G31" si="1">E2*F2</f>
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>9</v>
@@ -857,21 +860,25 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="13" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" s="6">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="D5" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E5" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F5" s="9"/>
+        <v>4.1999999999999993</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1</v>
+      </c>
       <c r="G5" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.1999999999999993</v>
       </c>
       <c r="H5" s="17">
         <v>1</v>
@@ -1022,7 +1029,7 @@
       </c>
       <c r="H11" s="30">
         <f>I5/SUM(G2:G31)</f>
-        <v>0.35680363411108817</v>
+        <v>0.42656134287830166</v>
       </c>
       <c r="I11" s="31"/>
     </row>

</xml_diff>